<commit_message>
Refresh the E2E screenshots and reports from today's verification run
Regenerated by the live runs behind the previous commit — the fixes
simulation's own screenshots plus the suites that re-exported their
workbooks. No source changes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/accessory-return-returns-page/downloaded-returns-report.xlsx
+++ b/e2e-screenshots/accessory-return-returns-page/downloaded-returns-report.xlsx
@@ -81,7 +81,7 @@
     <t>Carriage costed from</t>
   </si>
   <si>
-    <t>2026-08-02</t>
+    <t>2026-08-05</t>
   </si>
   <si>
     <t>Uncosted (pre-tracking) returns</t>
@@ -756,7 +756,7 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
-        <v>46236.5</v>
+        <v>46239.5</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>13</v>
@@ -774,7 +774,7 @@
         <v>13</v>
       </c>
       <c r="G2" s="3">
-        <v>46236.5</v>
+        <v>46239.5</v>
       </c>
       <c r="H2" s="6">
         <v>26.97</v>

</xml_diff>

<commit_message>
Refresh e2e screenshots from the in-progress full sweep
Churn from running the whole e2e suite against the archive-enabled build.
Committed as the sweep goes; the remaining scripts' shots follow when it
finishes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/accessory-return-returns-page/downloaded-returns-report.xlsx
+++ b/e2e-screenshots/accessory-return-returns-page/downloaded-returns-report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="51">
   <si>
     <t>Period</t>
   </si>
@@ -81,7 +81,7 @@
     <t>Carriage costed from</t>
   </si>
   <si>
-    <t>2026-08-11</t>
+    <t>2026-09-05</t>
   </si>
   <si>
     <t>Uncosted (pre-tracking) returns</t>
@@ -133,6 +133,12 @@
   </si>
   <si>
     <t>Postage Loss £</t>
+  </si>
+  <si>
+    <t>Fee Loss £</t>
+  </si>
+  <si>
+    <t>Stock In Date</t>
   </si>
   <si>
     <t>USB-C 20W Charger</t>
@@ -701,10 +707,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>24</v>
       </c>
@@ -753,16 +759,22 @@
       <c r="P1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q1" t="s">
+        <v>40</v>
+      </c>
+      <c r="R1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
-        <v>46245.5</v>
+        <v>46270.5</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>13</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>13</v>
@@ -774,7 +786,7 @@
         <v>13</v>
       </c>
       <c r="G2" s="3">
-        <v>46245.5</v>
+        <v>46270.5</v>
       </c>
       <c r="H2" s="6">
         <v>26.97</v>
@@ -783,13 +795,13 @@
         <v>10</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M2" s="5" t="s">
         <v>13</v>
@@ -803,6 +815,8 @@
       <c r="P2" s="6">
         <v>15.12</v>
       </c>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -823,16 +837,16 @@
         <v>26</v>
       </c>
       <c r="C1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G1" t="s">
         <v>36</v>
@@ -840,7 +854,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Anchor the downloadReport call sites too
The same "Import Inventory Report" / "Import Sales Report" collision, passed
as a regex argument rather than written inline, so the earlier anchoring
pass did not reach it. These scripts opened the importer, and its z-[80]
backdrop then swallowed every later click.

  e2eAccessoryReturnViaReturnsPage  24 -> 29/29
  e2eAccessorySellAndFixes          14 -> 18/18
  e2eReturnsMenuAndDeviceCatalog     8 -> 13/13
  e2eBulkSale40                     12/12 in 900s (TIMED OUT) -> 15/15 in 117s

That last one is the same bug wearing a different face: its report click sits
near the end, so instead of failing it sat on the intercepted click until the
runner's 900s timeout killed it — fifteen minutes of every sweep, with every
assertion already passed.

Suite total 757/780 -> 774/797.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/accessory-return-returns-page/downloaded-returns-report.xlsx
+++ b/e2e-screenshots/accessory-return-returns-page/downloaded-returns-report.xlsx
@@ -81,7 +81,7 @@
     <t>Carriage costed from</t>
   </si>
   <si>
-    <t>2026-09-05</t>
+    <t>2026-09-09</t>
   </si>
   <si>
     <t>Uncosted (pre-tracking) returns</t>
@@ -768,7 +768,7 @@
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
-        <v>46270.5</v>
+        <v>46274.5</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>13</v>
@@ -786,7 +786,7 @@
         <v>13</v>
       </c>
       <c r="G2" s="3">
-        <v>46270.5</v>
+        <v>46274.5</v>
       </c>
       <c r="H2" s="6">
         <v>26.97</v>

</xml_diff>